<commit_message>
docs(test-cases): rewrite Steps as numbered user-friendly steps
Each manual case now lists 1/2/3 UI-level steps (what a tester actually
does) instead of a single API-centric line. Excel cells keep real line
breaks; markdown uses <br>.
</commit_message>
<xml_diff>
--- a/TEST_CASES.xlsx
+++ b/TEST_CASES.xlsx
@@ -550,7 +550,9 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>POST /api/auth/login body {username, password} ถูกต้อง</t>
+          <t>1. เปิดหน้า /login
+2. กรอก username และ password ที่มีในระบบ
+3. กดปุ่ม Login</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
@@ -590,7 +592,9 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>POST ด้วย password ผิด</t>
+          <t>1. เปิดหน้า /login
+2. กรอก username ถูก แต่ password ผิด
+3. กดปุ่ม Login</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -630,7 +634,9 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>POST ด้วย username ที่ไม่มี</t>
+          <t>1. เปิดหน้า /login
+2. กรอก username ที่ไม่มีในระบบ
+3. กดปุ่ม Login</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -670,7 +676,9 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>เปิด /dobot, /camera, /drawing, /settings, /dashboard</t>
+          <t>1. ล้าง token (logout หรือลบ localStorage)
+2. พิมพ์ URL เช่น /dobot แล้วกด Enter
+3. ทำซ้ำกับ /camera, /drawing, /settings, /dashboard</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -710,7 +718,8 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>เปิดหน้า protected</t>
+          <t>1. ใช้ token ที่หมดอายุแล้ว
+2. เปิดหน้า protected เช่น /dobot</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -750,7 +759,8 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>GET /api/auth/me</t>
+          <t>1. ใส่ token ที่ผิดรูปแบบ
+2. เปิดหน้า protected หรือเรียก /api/auth/me</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -790,7 +800,8 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>GET /api/auth/me</t>
+          <t>1. ไม่แนบ header Authorization
+2. เรียก GET /api/auth/me</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
@@ -830,7 +841,8 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>GET /api/auth/me พร้อม Bearer</t>
+          <t>1. Login ให้ได้ token
+2. เรียก GET /api/auth/me พร้อม Bearer token</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -870,7 +882,8 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>POST /api/auth/register ไม่มี token</t>
+          <t>1. ไม่ login (ไม่มี token)
+2. เรียก POST /api/auth/register</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
@@ -910,7 +923,8 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>POST register username="a"</t>
+          <t>1. Login ก่อน
+2. เรียก register ด้วย username ยาว 1 ตัวอักษร</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -950,7 +964,8 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>POST register password="x"</t>
+          <t>1. Login ก่อน
+2. เรียก register ด้วย password ยาว 1 ตัวอักษร</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
@@ -990,7 +1005,9 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>POST register username="admin"</t>
+          <t>1. Login ก่อน
+2. ให้มี user ชื่อ admin อยู่แล้ว
+3. เรียก register ด้วย username admin</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -1030,7 +1047,8 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>POST register user ใหม่ (username≥2, password≥4)</t>
+          <t>1. Login ก่อน
+2. เรียก register ด้วย username ≥2 ตัว และ password ≥4 ตัว ที่ยังไม่มี</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
@@ -1070,7 +1088,9 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>กด Logout</t>
+          <t>1. Login อยู่
+2. กดปุ่ม Logout
+3. สังเกตว่าเด้งกลับหน้า /login</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
@@ -1110,7 +1130,9 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>เรียก apiFetch</t>
+          <t>1. ให้มี token ใน localStorage
+2. เรียก apiFetch ไป endpoint ที่ต้อง auth
+3. ดู header ของ request ที่ส่งออก</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
@@ -1150,7 +1172,9 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>apiFetch(url,{headers:{Authorization:'Bearer x'}})</t>
+          <t>1. ให้มี token
+2. เรียก apiFetch พร้อม header Authorization ที่ส่งมาเอง
+3. ดู header ที่ส่งออกจริง</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1190,7 +1214,9 @@
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>apiFetch (GET)</t>
+          <t>1. ให้ server ตอบ 500 ครั้งแรก แล้ว 200
+2. เรียก apiFetch (GET)
+3. นับจำนวนครั้งที่ fetch ถูกเรียก</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
@@ -1230,7 +1256,8 @@
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>เกิด 5xx</t>
+          <t>1. ทำให้เกิด response 5xx
+2. สังเกตแบนเนอร์แจ้งเตือนด้านบนจอ</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1270,7 +1297,9 @@
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>เรียก endpoint ที่คืน 401</t>
+          <t>1. อยู่หน้า /dobot (มี token)
+2. เรียก endpoint ที่ตอบ 401
+3. สังเกตว่าเด้งไป /login</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
@@ -1310,7 +1339,8 @@
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>POST /api/auth/login คืน 401</t>
+          <t>1. เรียก /api/auth/login ที่ตอบ 401
+2. สังเกตว่าไม่มีการเด้งไป /login</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1350,7 +1380,8 @@
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>ให้เกิด 5xx แล้วรอ 8 วิ</t>
+          <t>1. ทำให้เกิด 5xx
+2. รอ 8 วินาที (หรือกดปุ่ม ✕ ปิด)</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
@@ -1390,7 +1421,8 @@
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>เปิด /dashboard</t>
+          <t>1. Login
+2. เปิดเมนู Dashboard</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1430,7 +1462,9 @@
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>เฝ้าหน้า 2–3 วิ</t>
+          <t>1. เชื่อมต่อหุ่นจริง
+2. เปิด Dashboard
+3. เฝ้าดู 2–3 วินาที</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
@@ -1470,7 +1504,9 @@
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>เปิด dashboard</t>
+          <t>1. ปิดหุ่น/กล้อง
+2. เปิด Dashboard
+3. ดูสถานะว่ารอ/ตัดการเชื่อมต่อ</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
@@ -1510,7 +1546,9 @@
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>เลือกแกน X, step=1, กด + / −</t>
+          <t>1. เชื่อมต่อหุ่น
+2. เลือกแกน X และ step = 1
+3. กดปุ่ม + แล้วกดปุ่ม −</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
@@ -1550,7 +1588,9 @@
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>เลือก J1, step, กด + / −</t>
+          <t>1. เชื่อมต่อหุ่น
+2. เลือกข้อต่อ J1
+3. กดปุ่ม + / −</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
@@ -1590,7 +1630,9 @@
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>เปลี่ยนค่า step แล้ว jog</t>
+          <t>1. เลือก step = 0.1
+2. กด jog แล้ววัดระยะที่ขยับ
+3. ทำซ้ำกับ step 1, 5, 10</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
@@ -1630,7 +1672,8 @@
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>ดูแถบพิกัด</t>
+          <t>1. เชื่อมต่อหุ่น
+2. ดูแถบพิกัด (X/Y/Z/RX/RY/RZ + J1–J6) แบบสด</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
@@ -1670,7 +1713,8 @@
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>ดูโมเดล 3D</t>
+          <t>1. เปิดหน้า /dobot
+2. เทียบท่าทางโมเดล 3D กับพิกัดจริง</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
@@ -1710,7 +1754,9 @@
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>ลากลูกบอลปลายแขน</t>
+          <t>1. เปิด 3D viewer
+2. ลากลูกบอลสีส้มที่ปลายแขน
+3. สังเกตว่าทุกข้อต่อขยับตาม</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
@@ -1750,7 +1796,9 @@
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>กดปุ่ม Home</t>
+          <t>1. เชื่อมต่อหุ่น
+2. กดปุ่ม Home
+3. รอหุ่นเคลื่อนไปตำแหน่ง HOME</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
@@ -1790,7 +1838,9 @@
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>กดปุ่ม E-Stop</t>
+          <t>1. เริ่มให้มีการเคลื่อนที่ (jog/align/draw)
+2. กดปุ่ม E-Stop
+3. สังเกตว่าหุ่นหยุดทันที</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
@@ -1830,7 +1880,8 @@
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>POST /api/map/error</t>
+          <t>1. ทำให้หุ่นเข้า error state
+2. กดปุ่ม Clear error</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
@@ -1870,7 +1921,9 @@
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>กดปุ่มเชื่อมต่อ/init/start cam</t>
+          <t>1. กดปุ่ม Connect
+2. กดปุ่ม Init
+3. กดปุ่ม Start Camera</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
@@ -1910,7 +1963,9 @@
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>ส่งคำสั่งผ่าน CLI</t>
+          <t>1. เชื่อมต่อหุ่น
+2. พิมพ์คำสั่งในช่อง CLI
+3. กดส่ง แล้วดูผลลัพธ์</t>
         </is>
       </c>
       <c r="G36" s="3" t="inlineStr">
@@ -1950,7 +2005,8 @@
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>เปิด /camera</t>
+          <t>1. เปิดหน้า /camera
+2. ดูภาพสดจากกล้อง</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
@@ -1990,7 +2046,9 @@
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>กด Capture</t>
+          <t>1. เปิดหน้า /camera
+2. กดปุ่ม Capture
+3. ตรวจว่ามีไฟล์ภาพ JPEG</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
@@ -2030,7 +2088,9 @@
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>กดปุ่มโหมด</t>
+          <t>1. เปิดหน้า /camera
+2. กดสลับโหมด rgb / gray / depth
+3. สังเกตภาพเปลี่ยนตามโหมด</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr">
@@ -2070,7 +2130,8 @@
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>กด toggle</t>
+          <t>1. กดปุ่ม toggle โหมด
+2. สังเกตว่าโหมดวนไปตามลำดับ</t>
         </is>
       </c>
       <c r="G40" s="3" t="inlineStr">
@@ -2110,7 +2171,9 @@
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>เปิดหน้า/กด scan</t>
+          <t>1. เปิดหน้า /camera
+2. กด Scan หรือดูรายการกล้อง
+3. เห็น serial ของกล้องทั้งหมด</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr">
@@ -2150,7 +2213,8 @@
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>เปิด stream2</t>
+          <t>1. ต่อกล้อง D455 2 ตัว
+2. เปิด stream ของกล้องตัวที่ 2</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr">
@@ -2190,7 +2254,9 @@
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>กด Swap View</t>
+          <t>1. ต่อกล้อง 2 ตัว
+2. กดปุ่ม Swap View
+3. ภาพกล้องหลัก/รองสลับกัน</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
@@ -2230,7 +2296,9 @@
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>POST /api/camera/select</t>
+          <t>1. ต่อกล้องหลายตัว
+2. เลือกกล้องหลักจากรายการ
+3. ภาพหลักเปลี่ยนตามที่เลือก</t>
         </is>
       </c>
       <c r="G44" s="3" t="inlineStr">
@@ -2270,7 +2338,8 @@
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>GET /api/camera/snapshot2</t>
+          <t>1. ต่อกล้อง 2 ตัว
+2. กด Capture ของกล้องตัวที่ 2</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
@@ -2310,7 +2379,9 @@
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>กด Capture</t>
+          <t>1. mark จุดบนภาพ
+2. กด Capture
+3. ตรวจว่าจุดที่ mark ปรากฏในภาพที่บันทึก</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
@@ -2350,7 +2421,9 @@
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>POST /api/map/grid/size rows/cols</t>
+          <t>1. เปิดหน้า /drawing
+2. ไปแท็บ Grid
+3. ตั้งค่า rows/cols (ไม่เกิน 7×7)</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr">
@@ -2390,7 +2463,9 @@
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>กด Mark ทีละมุม</t>
+          <t>1. jog หุ่นไปที่จุดมุม
+2. กดปุ่ม Mark
+3. ทำซ้ำจนครบทุกจุดใน grid</t>
         </is>
       </c>
       <c r="G48" s="3" t="inlineStr">
@@ -2430,7 +2505,9 @@
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>ดูผล validate</t>
+          <t>1. mark จุดให้ครบ
+2. ดูผลการ validate
+3. เตือนเมื่อ span เล็กเกินไป หรือ rmse &gt; 3mm</t>
         </is>
       </c>
       <c r="G49" s="3" t="inlineStr">
@@ -2470,7 +2547,9 @@
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>กด Autofill</t>
+          <t>1. mark จุดแล้ว
+2. กดปุ่ม Autofill Z
+3. ดูค่า Z ถูกเติมตามพื้นผิว</t>
         </is>
       </c>
       <c r="G50" s="3" t="inlineStr">
@@ -2510,7 +2589,8 @@
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>กด Reset</t>
+          <t>1. มี grid ที่สอนไว้
+2. กดปุ่ม Reset grid</t>
         </is>
       </c>
       <c r="G51" s="3" t="inlineStr">
@@ -2550,7 +2630,9 @@
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>POST /api/map/grid/restore</t>
+          <t>1. มี pose ของ grid ครบ
+2. เรียก /api/map/grid/restore
+3. grid กลับมาโดยไม่ต้องสอนใหม่</t>
         </is>
       </c>
       <c r="G52" s="3" t="inlineStr">
@@ -2590,7 +2672,8 @@
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>สังเกตหลังวาด</t>
+          <t>1. วาดจนจบงาน
+2. สังเกตว่าหัวหุ่นกลับไปจุดเริ่ม</t>
         </is>
       </c>
       <c r="G53" s="3" t="inlineStr">
@@ -2630,7 +2713,9 @@
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>วาดบน canvas แล้ว Send</t>
+          <t>1. สอน grid ให้ครบ
+2. วาดเส้นบน canvas
+3. กดปุ่ม Send แล้วดูหุ่นวาดตามเส้น</t>
         </is>
       </c>
       <c r="G54" s="3" t="inlineStr">
@@ -2670,7 +2755,9 @@
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>กด Stop</t>
+          <t>1. เริ่มวาด (กำลังเคลื่อนที่)
+2. กดปุ่ม Stop
+3. หยุดทันที</t>
         </is>
       </c>
       <c r="G55" s="3" t="inlineStr">
@@ -2710,7 +2797,9 @@
       </c>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>ส่งหลาย stroke</t>
+          <t>1. วาด 2 รูปคนละตำแหน่ง
+2. กด Send
+3. สังเกตการยกหัวก่อนข้ามไปรูปถัดไป</t>
         </is>
       </c>
       <c r="G56" s="3" t="inlineStr">
@@ -2750,7 +2839,9 @@
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>กดจุดบนภาพ</t>
+          <t>1. เชื่อมต่อหุ่น
+2. กดจุดบนภาพ (โหมด goto/point)
+3. หุ่นไปยังจุดนั้น</t>
         </is>
       </c>
       <c r="G57" s="3" t="inlineStr">
@@ -2790,7 +2881,9 @@
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>เปลี่ยน frame (User/Tool)</t>
+          <t>1. เชื่อมต่อหุ่น
+2. เปลี่ยน frame เป็น User/Tool
+3. สังเกตพิกัดเปลี่ยนตาม frame</t>
         </is>
       </c>
       <c r="G58" s="3" t="inlineStr">
@@ -2830,7 +2923,9 @@
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>กดแท็บ Align / Grid / Jog / All</t>
+          <t>1. เปิดหน้า /drawing
+2. กดแท็บ Align, Grid, Jog, All สลับไปมา
+3. สังเกตว่าเนื้อหา panel เปลี่ยนตามแท็บ</t>
         </is>
       </c>
       <c r="G59" s="3" t="inlineStr">
@@ -2870,7 +2965,9 @@
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>กดปุ่ม Fold</t>
+          <t>1. เปิดหน้า /drawing
+2. กดปุ่ม Fold
+3. สังเกต panel ย่อ และกดอีกครั้งเพื่อกาง</t>
         </is>
       </c>
       <c r="G60" s="3" t="inlineStr">
@@ -2910,7 +3007,9 @@
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>ดู pills ด้านบน panel</t>
+          <t>1. เชื่อมต่อหุ่น
+2. ดู status pills บน panel
+3. สถานะ/โหมดหุ่นแสดงถูกต้อง</t>
         </is>
       </c>
       <c r="G61" s="3" t="inlineStr">
@@ -2950,7 +3049,9 @@
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>กด Connect / Init / CamStart / Heatmap</t>
+          <t>1. เชื่อมต่อหุ่น
+2. กด Connect, Init, CamStart, Heatmap ทีละปุ่ม
+3. endpoint ถูกเรียกตามปุ่ม</t>
         </is>
       </c>
       <c r="G62" s="3" t="inlineStr">
@@ -2990,7 +3091,9 @@
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>เปลี่ยน rows/cols ในแท็บ Grid</t>
+          <t>1. ไปแท็บ Grid
+2. เปลี่ยนค่า rows/cols
+3. ขนาด grid อัปเดต (ไม่เกิน 7×7)</t>
         </is>
       </c>
       <c r="G63" s="3" t="inlineStr">
@@ -3030,7 +3133,9 @@
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>ดูการ์ด Cells Matrix</t>
+          <t>1. mark grid ครบ
+2. ดูการ์ด Cells Matrix &amp; Shape
+3. เห็น preview รูปร่าง grid ตามที่สอน</t>
         </is>
       </c>
       <c r="G64" s="3" t="inlineStr">
@@ -3070,7 +3175,9 @@
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>ใช้ปุ่ม jog ในแท็บ Jog</t>
+          <t>1. เชื่อมต่อหุ่น
+2. ไปแท็บ Jog
+3. กดปุ่ม jog ตามแกน/step</t>
         </is>
       </c>
       <c r="G65" s="3" t="inlineStr">
@@ -3110,7 +3217,9 @@
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>ปรับ step/speed</t>
+          <t>1. ปรับค่า step/speed
+2. กด jog
+3. ระยะ/ความเร็วสอดคล้องกับค่าที่ตั้ง</t>
         </is>
       </c>
       <c r="G66" s="3" t="inlineStr">
@@ -3150,7 +3259,9 @@
       </c>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>กด Align ในแท็บ Align</t>
+          <t>1. mark 4 มุม
+2. ไปแท็บ Align
+3. กดปุ่ม Align</t>
         </is>
       </c>
       <c r="G67" s="3" t="inlineStr">
@@ -3190,7 +3301,8 @@
       </c>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>เปลี่ยน frame</t>
+          <t>1. เชื่อมต่อหุ่น
+2. เปลี่ยน coordinate frame ใน panel</t>
         </is>
       </c>
       <c r="G68" s="3" t="inlineStr">
@@ -3230,7 +3342,9 @@
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>สังเกตตำแหน่ง viewer</t>
+          <t>1. เปิดหน้า /drawing
+2. สังเกตตำแหน่ง 3D viewer
+3. viewer อยู่มุมล่างซ้าย</t>
         </is>
       </c>
       <c r="G69" s="3" t="inlineStr">
@@ -3270,7 +3384,9 @@
       </c>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>กด Start Align</t>
+          <t>1. mark 4 จุด และเปิดกล้อง depth
+2. กดปุ่ม Start Align
+3. หุ่นเริ่มหมุนเพื่อปรับระนาบ</t>
         </is>
       </c>
       <c r="G70" s="3" t="inlineStr">
@@ -3310,7 +3426,9 @@
       </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>เฝ้า status</t>
+          <t>1. เริ่ม align
+2. เฝ้าดูค่า tilt ใน status
+3. หยุดเองเมื่อ tilt ≤ ALIGN_TOL_DEG</t>
         </is>
       </c>
       <c r="G71" s="3" t="inlineStr">
@@ -3350,7 +3468,8 @@
       </c>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t>กด Stop</t>
+          <t>1. ระหว่าง align
+2. กดปุ่ม Stop</t>
         </is>
       </c>
       <c r="G72" s="3" t="inlineStr">
@@ -3390,7 +3509,9 @@
       </c>
       <c r="F73" s="3" t="inlineStr">
         <is>
-          <t>เริ่ม align</t>
+          <t>1. mark จุดที่ tracker ยังไม่ lock
+2. เริ่ม align
+3. มีการลองใหม่สั้น ๆ แล้วแจ้ง points not locked</t>
         </is>
       </c>
       <c r="G73" s="3" t="inlineStr">
@@ -3430,7 +3551,8 @@
       </c>
       <c r="F74" s="3" t="inlineStr">
         <is>
-          <t>กด Clear</t>
+          <t>1. มีจุด mark อยู่
+2. กดปุ่ม Clear points</t>
         </is>
       </c>
       <c r="G74" s="3" t="inlineStr">
@@ -3470,7 +3592,8 @@
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>กด toggle</t>
+          <t>1. เปิดกล้อง depth
+2. กดปุ่ม toggle heatmap</t>
         </is>
       </c>
       <c r="G75" s="3" t="inlineStr">
@@ -3510,7 +3633,9 @@
       </c>
       <c r="F76" s="3" t="inlineStr">
         <is>
-          <t>POST /api/map/move_to</t>
+          <t>1. เชื่อมต่อหุ่น
+2. เรียก move_to ด้วย pose เป้าหมาย
+3. หุ่นเคลื่อนไปยัง pose นั้น</t>
         </is>
       </c>
       <c r="G76" s="3" t="inlineStr">
@@ -3550,7 +3675,9 @@
       </c>
       <c r="F77" s="3" t="inlineStr">
         <is>
-          <t>POST /api/map/move_sequence</t>
+          <t>1. ตั้งลำดับ waypoint
+2. เรียก move_sequence
+3. หุ่นวิ่งตามลำดับ</t>
         </is>
       </c>
       <c r="G77" s="3" t="inlineStr">
@@ -3590,7 +3717,8 @@
       </c>
       <c r="F78" s="3" t="inlineStr">
         <is>
-          <t>POST /api/map/move_sequence/stop</t>
+          <t>1. เริ่ม move sequence
+2. กดปุ่มหยุด sequence</t>
         </is>
       </c>
       <c r="G78" s="3" t="inlineStr">
@@ -3630,7 +3758,9 @@
       </c>
       <c r="F79" s="3" t="inlineStr">
         <is>
-          <t>POST {axis,direction,step}</t>
+          <t>1. เชื่อมต่อหุ่น
+2. ส่ง {axis, direction, step}
+3. หุ่นขยับตามที่สั่ง</t>
         </is>
       </c>
       <c r="G79" s="3" t="inlineStr">
@@ -3670,7 +3800,8 @@
       </c>
       <c r="F80" s="3" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>1. เชื่อมต่อหุ่น
+2. เรียก /api/robot/emergency-stop</t>
         </is>
       </c>
       <c r="G80" s="3" t="inlineStr">
@@ -3710,7 +3841,9 @@
       </c>
       <c r="F81" s="3" t="inlineStr">
         <is>
-          <t>เปิด /settings</t>
+          <t>1. Login
+2. เปิดหน้า /settings
+3. ดูค่าที่โหลดมาแสดง</t>
         </is>
       </c>
       <c r="G81" s="3" t="inlineStr">
@@ -3750,7 +3883,9 @@
       </c>
       <c r="F82" s="3" t="inlineStr">
         <is>
-          <t>PUT /api/settings</t>
+          <t>1. เปิดหน้า /settings
+2. แก้ค่า แล้วกดบันทึก
+3. โหลดใหม่แล้วค่ายังอยู่</t>
         </is>
       </c>
       <c r="G82" s="3" t="inlineStr">
@@ -3790,7 +3925,9 @@
       </c>
       <c r="F83" s="3" t="inlineStr">
         <is>
-          <t>PUT /api/settings/{key}</t>
+          <t>1. แก้ค่าเฉพาะ key เดียว
+2. บันทึก
+3. key อื่นไม่เปลี่ยน</t>
         </is>
       </c>
       <c r="G83" s="3" t="inlineStr">
@@ -3830,7 +3967,8 @@
       </c>
       <c r="F84" s="3" t="inlineStr">
         <is>
-          <t>POST /api/devices/relay/toggle</t>
+          <t>1. ตั้ง Blynk token
+2. กดปุ่ม toggle relay</t>
         </is>
       </c>
       <c r="G84" s="3" t="inlineStr">
@@ -3870,7 +4008,8 @@
       </c>
       <c r="F85" s="3" t="inlineStr">
         <is>
-          <t>GET /api/devices/relay/state</t>
+          <t>1. เปิดหน้า Devices
+2. ดูสถานะ relay ปัจจุบัน</t>
         </is>
       </c>
       <c r="G85" s="3" t="inlineStr">
@@ -3910,7 +4049,8 @@
       </c>
       <c r="F86" s="3" t="inlineStr">
         <is>
-          <t>GET /api/devices/relay/history</t>
+          <t>1. เปิดหน้า Devices
+2. ดูประวัติการสั่ง relay</t>
         </is>
       </c>
       <c r="G86" s="3" t="inlineStr">
@@ -3950,7 +4090,9 @@
       </c>
       <c r="F87" s="3" t="inlineStr">
         <is>
-          <t>GET /api/devices/ping</t>
+          <t>1. เปิดหน้า Devices
+2. กดปุ่ม ping
+3. แสดงสถานะเข้าถึงได้/ไม่ได้</t>
         </is>
       </c>
       <c r="G87" s="3" t="inlineStr">
@@ -3990,7 +4132,9 @@
       </c>
       <c r="F88" s="3" t="inlineStr">
         <is>
-          <t>เรียก /api/map/status ไม่มี token</t>
+          <t>1. ไม่แนบ token
+2. เรียก /api/map/status
+3. สังเกตว่าได้ 401 (ยกเว้น /api/auth/*)</t>
         </is>
       </c>
       <c r="G88" s="3" t="inlineStr">
@@ -4030,7 +4174,9 @@
       </c>
       <c r="F89" s="3" t="inlineStr">
         <is>
-          <t>ยิงจาก origin ที่อนุญาต/ไม่อนุญาต</t>
+          <t>1. ตั้ง ALLOWED_ORIGINS
+2. ยิงจาก origin ที่อนุญาต และที่ไม่อนุญาต
+3. เทียบผล</t>
         </is>
       </c>
       <c r="G89" s="3" t="inlineStr">
@@ -4070,7 +4216,8 @@
       </c>
       <c r="F90" s="3" t="inlineStr">
         <is>
-          <t>preflight OPTIONS</t>
+          <t>1. ส่ง preflight OPTIONS ไป endpoint
+2. สังเกตว่าไม่ถูกบล็อกด้วย 401</t>
         </is>
       </c>
       <c r="G90" s="3" t="inlineStr">
@@ -4110,7 +4257,8 @@
       </c>
       <c r="F91" s="3" t="inlineStr">
         <is>
-          <t>GET /</t>
+          <t>1. เรียก GET /
+2. ได้ข้อความ Robot Arm API is running</t>
         </is>
       </c>
       <c r="G91" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Add manual test results and new-feature test cases (scan/align/mesh/logs); ignore Excel lock files
</commit_message>
<xml_diff>
--- a/TEST_CASES.xlsx
+++ b/TEST_CASES.xlsx
@@ -561,8 +561,16 @@
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>login 200 + access_token</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -603,8 +611,16 @@
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr"/>
-      <c r="I3" s="2" t="inlineStr"/>
-      <c r="J3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>401 Invalid credentials</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -645,8 +661,16 @@
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>401</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -687,8 +711,16 @@
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr"/>
-      <c r="I5" s="2" t="inlineStr"/>
-      <c r="J5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Needs Browser</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>UI redirect (RequireAuth)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -728,8 +760,16 @@
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr"/>
-      <c r="I6" s="2" t="inlineStr"/>
-      <c r="J6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>expired token -&gt; 401</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -769,8 +809,16 @@
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr"/>
-      <c r="I7" s="2" t="inlineStr"/>
-      <c r="J7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>bad token -&gt; 401</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -810,8 +858,16 @@
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr"/>
-      <c r="I8" s="2" t="inlineStr"/>
-      <c r="J8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>no header -&gt; 401</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -851,8 +907,16 @@
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr"/>
-      <c r="I9" s="2" t="inlineStr"/>
-      <c r="J9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>/me 200 + {id, username}</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -892,8 +956,16 @@
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr"/>
-      <c r="I10" s="2" t="inlineStr"/>
-      <c r="J10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>no token -&gt; 401</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -933,8 +1005,16 @@
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr"/>
-      <c r="I11" s="2" t="inlineStr"/>
-      <c r="J11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>username 1 char -&gt; 400</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -974,8 +1054,16 @@
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr"/>
-      <c r="I12" s="2" t="inlineStr"/>
-      <c r="J12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>password 1 char -&gt; 400</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1016,8 +1104,16 @@
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr"/>
-      <c r="I13" s="2" t="inlineStr"/>
-      <c r="J13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>dup admin -&gt; 409</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1057,8 +1153,16 @@
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr"/>
-      <c r="I14" s="2" t="inlineStr"/>
-      <c r="J14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>register 200 + token</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1099,8 +1203,16 @@
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr"/>
-      <c r="I15" s="2" t="inlineStr"/>
-      <c r="J15" s="2" t="inlineStr"/>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Needs Browser</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>UI logout button</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1141,8 +1253,16 @@
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr"/>
-      <c r="I16" s="2" t="inlineStr"/>
-      <c r="J16" s="2" t="inlineStr"/>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>covered by FE-01 auto</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1183,8 +1303,16 @@
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr"/>
-      <c r="I17" s="2" t="inlineStr"/>
-      <c r="J17" s="2" t="inlineStr"/>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>covered by FE-01 auto</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1225,8 +1353,16 @@
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr"/>
-      <c r="I18" s="2" t="inlineStr"/>
-      <c r="J18" s="2" t="inlineStr"/>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>covered by FE-02 auto (retry)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1266,8 +1402,16 @@
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr"/>
-      <c r="I19" s="2" t="inlineStr"/>
-      <c r="J19" s="2" t="inlineStr"/>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>covered by FE-03 auto (banner)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1308,8 +1452,16 @@
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr"/>
-      <c r="I20" s="2" t="inlineStr"/>
-      <c r="J20" s="2" t="inlineStr"/>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>covered by FE-02 auto (401 redirect)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1349,8 +1501,16 @@
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr"/>
-      <c r="I21" s="2" t="inlineStr"/>
-      <c r="J21" s="2" t="inlineStr"/>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>covered by FE-02 auto</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1390,8 +1550,16 @@
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr"/>
-      <c r="I22" s="2" t="inlineStr"/>
-      <c r="J22" s="2" t="inlineStr"/>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>covered by FE-03 auto (auto-hide)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1431,8 +1599,16 @@
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr"/>
-      <c r="I23" s="2" t="inlineStr"/>
-      <c r="J23" s="2" t="inlineStr"/>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>status 200, robot connected=True</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1473,8 +1649,16 @@
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr"/>
-      <c r="I24" s="2" t="inlineStr"/>
-      <c r="J24" s="2" t="inlineStr"/>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>API poll 200; visual poll ต้องการ browser</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1515,8 +1699,16 @@
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr"/>
-      <c r="I25" s="2" t="inlineStr"/>
-      <c r="J25" s="2" t="inlineStr"/>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>Needs Rig</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>ต้องปิดหุ่น/กล้องจริง</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1557,8 +1749,16 @@
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr"/>
-      <c r="I26" s="2" t="inlineStr"/>
-      <c r="J26" s="2" t="inlineStr"/>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>Needs Rig</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>jog = หุ่นขยับ ต้องดูจริง</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1599,8 +1799,16 @@
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr"/>
-      <c r="I27" s="2" t="inlineStr"/>
-      <c r="J27" s="2" t="inlineStr"/>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>Needs Rig</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>jog joint = หุ่นขยับ</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1641,8 +1849,16 @@
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr"/>
-      <c r="I28" s="2" t="inlineStr"/>
-      <c r="J28" s="2" t="inlineStr"/>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>Needs Rig</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>วัดระยะจริง</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1682,8 +1898,16 @@
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr"/>
-      <c r="I29" s="2" t="inlineStr"/>
-      <c r="J29" s="2" t="inlineStr"/>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>status มี joints realtime (WS 20Hz)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1723,8 +1947,16 @@
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr"/>
-      <c r="I30" s="2" t="inlineStr"/>
-      <c r="J30" s="2" t="inlineStr"/>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>Needs Browser</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>3D viewer ต้องเห็นจริง</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1765,8 +1997,16 @@
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr"/>
-      <c r="I31" s="2" t="inlineStr"/>
-      <c r="J31" s="2" t="inlineStr"/>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>Needs Browser</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>IK drag UI</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1807,8 +2047,16 @@
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr"/>
-      <c r="I32" s="2" t="inlineStr"/>
-      <c r="J32" s="2" t="inlineStr"/>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>Needs Rig</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>Home = เคลื่อนหุ่น</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1849,8 +2097,16 @@
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr"/>
-      <c r="I33" s="2" t="inlineStr"/>
-      <c r="J33" s="2" t="inlineStr"/>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>emergency -&gt; emergency_stop_triggered</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1890,8 +2146,16 @@
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr"/>
-      <c r="I34" s="2" t="inlineStr"/>
-      <c r="J34" s="2" t="inlineStr"/>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>Needs Rig</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>ต้องทำให้หุ่น error ก่อน</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -1932,8 +2196,16 @@
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr"/>
-      <c r="I35" s="2" t="inlineStr"/>
-      <c r="J35" s="2" t="inlineStr"/>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>connect/init/camstart ทั้ง 3 ผ่าน</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1974,8 +2246,16 @@
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr"/>
-      <c r="I36" s="2" t="inlineStr"/>
-      <c r="J36" s="2" t="inlineStr"/>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>CLI 200, output กลับ (GetAngle)</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2015,8 +2295,16 @@
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr"/>
-      <c r="I37" s="2" t="inlineStr"/>
-      <c r="J37" s="2" t="inlineStr"/>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>MJPEG multipart 200 (กล้องหลักทำงาน)</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2057,8 +2345,16 @@
         </is>
       </c>
       <c r="H38" s="3" t="inlineStr"/>
-      <c r="I38" s="2" t="inlineStr"/>
-      <c r="J38" s="2" t="inlineStr"/>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>snapshot JPEG 161KB</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2099,8 +2395,16 @@
         </is>
       </c>
       <c r="H39" s="3" t="inlineStr"/>
-      <c r="I39" s="2" t="inlineStr"/>
-      <c r="J39" s="2" t="inlineStr"/>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>mode rgb -&gt; 200</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2140,8 +2444,16 @@
         </is>
       </c>
       <c r="H40" s="3" t="inlineStr"/>
-      <c r="I40" s="2" t="inlineStr"/>
-      <c r="J40" s="2" t="inlineStr"/>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>mode toggle -&gt; 200</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2182,8 +2494,16 @@
         </is>
       </c>
       <c r="H41" s="3" t="inlineStr"/>
-      <c r="I41" s="2" t="inlineStr"/>
-      <c r="J41" s="2" t="inlineStr"/>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>devices: D455 x2 (215122252229 / ...)</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -2223,8 +2543,16 @@
         </is>
       </c>
       <c r="H42" s="3" t="inlineStr"/>
-      <c r="I42" s="2" t="inlineStr"/>
-      <c r="J42" s="2" t="inlineStr"/>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>stream2 MJPEG 200 (กล้องรองทำงาน)</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -2265,8 +2593,16 @@
         </is>
       </c>
       <c r="H43" s="3" t="inlineStr"/>
-      <c r="I43" s="2" t="inlineStr"/>
-      <c r="J43" s="2" t="inlineStr"/>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>Needs Rig</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>swap กระทบ primary — ไม่รันรบกวน</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -2307,8 +2643,16 @@
         </is>
       </c>
       <c r="H44" s="3" t="inlineStr"/>
-      <c r="I44" s="2" t="inlineStr"/>
-      <c r="J44" s="2" t="inlineStr"/>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>Needs Rig</t>
+        </is>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>select primary — ไม่รันรบกวน</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -2348,8 +2692,16 @@
         </is>
       </c>
       <c r="H45" s="3" t="inlineStr"/>
-      <c r="I45" s="2" t="inlineStr"/>
-      <c r="J45" s="2" t="inlineStr"/>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>snapshot2 JPEG 88KB</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -2390,8 +2742,16 @@
         </is>
       </c>
       <c r="H46" s="3" t="inlineStr"/>
-      <c r="I46" s="2" t="inlineStr"/>
-      <c r="J46" s="2" t="inlineStr"/>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>Needs Browser</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>ต้อง mark บน UI</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -2432,8 +2792,16 @@
         </is>
       </c>
       <c r="H47" s="3" t="inlineStr"/>
-      <c r="I47" s="2" t="inlineStr"/>
-      <c r="J47" s="2" t="inlineStr"/>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>Needs Rig</t>
+        </is>
+      </c>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>grid บนหุ่นจริง</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -2474,8 +2842,16 @@
         </is>
       </c>
       <c r="H48" s="3" t="inlineStr"/>
-      <c r="I48" s="2" t="inlineStr"/>
-      <c r="J48" s="2" t="inlineStr"/>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>Needs Rig</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>jog+mark จริง</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -2516,7 +2892,11 @@
         </is>
       </c>
       <c r="H49" s="3" t="inlineStr"/>
-      <c r="I49" s="2" t="inlineStr"/>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>Needs Rig</t>
+        </is>
+      </c>
       <c r="J49" s="2" t="inlineStr"/>
     </row>
     <row r="50">
@@ -2558,7 +2938,11 @@
         </is>
       </c>
       <c r="H50" s="3" t="inlineStr"/>
-      <c r="I50" s="2" t="inlineStr"/>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>Needs Rig</t>
+        </is>
+      </c>
       <c r="J50" s="2" t="inlineStr"/>
     </row>
     <row r="51">
@@ -2599,7 +2983,11 @@
         </is>
       </c>
       <c r="H51" s="3" t="inlineStr"/>
-      <c r="I51" s="2" t="inlineStr"/>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>Needs Rig</t>
+        </is>
+      </c>
       <c r="J51" s="2" t="inlineStr"/>
     </row>
     <row r="52">
@@ -2641,7 +3029,11 @@
         </is>
       </c>
       <c r="H52" s="3" t="inlineStr"/>
-      <c r="I52" s="2" t="inlineStr"/>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>Needs Rig</t>
+        </is>
+      </c>
       <c r="J52" s="2" t="inlineStr"/>
     </row>
     <row r="53">
@@ -2682,7 +3074,11 @@
         </is>
       </c>
       <c r="H53" s="3" t="inlineStr"/>
-      <c r="I53" s="2" t="inlineStr"/>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>Needs Rig</t>
+        </is>
+      </c>
       <c r="J53" s="2" t="inlineStr"/>
     </row>
     <row r="54">
@@ -2724,8 +3120,16 @@
         </is>
       </c>
       <c r="H54" s="3" t="inlineStr"/>
-      <c r="I54" s="2" t="inlineStr"/>
-      <c r="J54" s="2" t="inlineStr"/>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>Needs Rig</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>วาดจริงต้องหุ่น+ปากกา</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -2766,7 +3170,11 @@
         </is>
       </c>
       <c r="H55" s="3" t="inlineStr"/>
-      <c r="I55" s="2" t="inlineStr"/>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>Needs Rig</t>
+        </is>
+      </c>
       <c r="J55" s="2" t="inlineStr"/>
     </row>
     <row r="56">
@@ -2808,7 +3216,11 @@
         </is>
       </c>
       <c r="H56" s="3" t="inlineStr"/>
-      <c r="I56" s="2" t="inlineStr"/>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>Needs Rig</t>
+        </is>
+      </c>
       <c r="J56" s="2" t="inlineStr"/>
     </row>
     <row r="57">
@@ -2850,8 +3262,16 @@
         </is>
       </c>
       <c r="H57" s="3" t="inlineStr"/>
-      <c r="I57" s="2" t="inlineStr"/>
-      <c r="J57" s="2" t="inlineStr"/>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t>Needs Rig</t>
+        </is>
+      </c>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
+          <t>goto/point = เคลื่อนหุ่น</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -2892,8 +3312,16 @@
         </is>
       </c>
       <c r="H58" s="3" t="inlineStr"/>
-      <c r="I58" s="2" t="inlineStr"/>
-      <c r="J58" s="2" t="inlineStr"/>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>Needs Rig</t>
+        </is>
+      </c>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>frame = เคลื่อนหุ่น</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -2934,8 +3362,16 @@
         </is>
       </c>
       <c r="H59" s="3" t="inlineStr"/>
-      <c r="I59" s="2" t="inlineStr"/>
-      <c r="J59" s="2" t="inlineStr"/>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t>Needs Browser</t>
+        </is>
+      </c>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
+          <t>UI tab</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -2976,8 +3412,16 @@
         </is>
       </c>
       <c r="H60" s="3" t="inlineStr"/>
-      <c r="I60" s="2" t="inlineStr"/>
-      <c r="J60" s="2" t="inlineStr"/>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>Needs Browser</t>
+        </is>
+      </c>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>UI fold</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -3018,8 +3462,16 @@
         </is>
       </c>
       <c r="H61" s="3" t="inlineStr"/>
-      <c r="I61" s="2" t="inlineStr"/>
-      <c r="J61" s="2" t="inlineStr"/>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
+          <t>Needs Browser</t>
+        </is>
+      </c>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>UI pills</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -3060,8 +3512,16 @@
         </is>
       </c>
       <c r="H62" s="3" t="inlineStr"/>
-      <c r="I62" s="2" t="inlineStr"/>
-      <c r="J62" s="2" t="inlineStr"/>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>Needs Browser</t>
+        </is>
+      </c>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>UI quick actions</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -3102,8 +3562,16 @@
         </is>
       </c>
       <c r="H63" s="3" t="inlineStr"/>
-      <c r="I63" s="2" t="inlineStr"/>
-      <c r="J63" s="2" t="inlineStr"/>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
+          <t>Needs Browser</t>
+        </is>
+      </c>
+      <c r="J63" s="2" t="inlineStr">
+        <is>
+          <t>UI grid setup</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -3144,7 +3612,11 @@
         </is>
       </c>
       <c r="H64" s="3" t="inlineStr"/>
-      <c r="I64" s="2" t="inlineStr"/>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>Needs Browser</t>
+        </is>
+      </c>
       <c r="J64" s="2" t="inlineStr"/>
     </row>
     <row r="65">
@@ -3186,7 +3658,11 @@
         </is>
       </c>
       <c r="H65" s="3" t="inlineStr"/>
-      <c r="I65" s="2" t="inlineStr"/>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>Needs Browser</t>
+        </is>
+      </c>
       <c r="J65" s="2" t="inlineStr"/>
     </row>
     <row r="66">
@@ -3228,7 +3704,11 @@
         </is>
       </c>
       <c r="H66" s="3" t="inlineStr"/>
-      <c r="I66" s="2" t="inlineStr"/>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>Needs Browser</t>
+        </is>
+      </c>
       <c r="J66" s="2" t="inlineStr"/>
     </row>
     <row r="67">
@@ -3270,8 +3750,16 @@
         </is>
       </c>
       <c r="H67" s="3" t="inlineStr"/>
-      <c r="I67" s="2" t="inlineStr"/>
-      <c r="J67" s="2" t="inlineStr"/>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t>Needs Rig</t>
+        </is>
+      </c>
+      <c r="J67" s="2" t="inlineStr">
+        <is>
+          <t>align = เคลื่อนหุ่น</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -3311,7 +3799,11 @@
         </is>
       </c>
       <c r="H68" s="3" t="inlineStr"/>
-      <c r="I68" s="2" t="inlineStr"/>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>Needs Browser</t>
+        </is>
+      </c>
       <c r="J68" s="2" t="inlineStr"/>
     </row>
     <row r="69">
@@ -3353,8 +3845,16 @@
         </is>
       </c>
       <c r="H69" s="3" t="inlineStr"/>
-      <c r="I69" s="2" t="inlineStr"/>
-      <c r="J69" s="2" t="inlineStr"/>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>Needs Browser</t>
+        </is>
+      </c>
+      <c r="J69" s="2" t="inlineStr">
+        <is>
+          <t>viewer ตำแหน่ง UI</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -3395,8 +3895,16 @@
         </is>
       </c>
       <c r="H70" s="3" t="inlineStr"/>
-      <c r="I70" s="2" t="inlineStr"/>
-      <c r="J70" s="2" t="inlineStr"/>
+      <c r="I70" s="2" t="inlineStr">
+        <is>
+          <t>Needs Rig</t>
+        </is>
+      </c>
+      <c r="J70" s="2" t="inlineStr">
+        <is>
+          <t>align = เคลื่อนหุ่น</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -3437,7 +3945,11 @@
         </is>
       </c>
       <c r="H71" s="3" t="inlineStr"/>
-      <c r="I71" s="2" t="inlineStr"/>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t>Needs Rig</t>
+        </is>
+      </c>
       <c r="J71" s="2" t="inlineStr"/>
     </row>
     <row r="72">
@@ -3478,7 +3990,11 @@
         </is>
       </c>
       <c r="H72" s="3" t="inlineStr"/>
-      <c r="I72" s="2" t="inlineStr"/>
+      <c r="I72" s="2" t="inlineStr">
+        <is>
+          <t>Needs Rig</t>
+        </is>
+      </c>
       <c r="J72" s="2" t="inlineStr"/>
     </row>
     <row r="73">
@@ -3520,7 +4036,11 @@
         </is>
       </c>
       <c r="H73" s="3" t="inlineStr"/>
-      <c r="I73" s="2" t="inlineStr"/>
+      <c r="I73" s="2" t="inlineStr">
+        <is>
+          <t>Needs Rig</t>
+        </is>
+      </c>
       <c r="J73" s="2" t="inlineStr"/>
     </row>
     <row r="74">
@@ -3561,7 +4081,11 @@
         </is>
       </c>
       <c r="H74" s="3" t="inlineStr"/>
-      <c r="I74" s="2" t="inlineStr"/>
+      <c r="I74" s="2" t="inlineStr">
+        <is>
+          <t>Needs Rig</t>
+        </is>
+      </c>
       <c r="J74" s="2" t="inlineStr"/>
     </row>
     <row r="75">
@@ -3602,8 +4126,16 @@
         </is>
       </c>
       <c r="H75" s="3" t="inlineStr"/>
-      <c r="I75" s="2" t="inlineStr"/>
-      <c r="J75" s="2" t="inlineStr"/>
+      <c r="I75" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J75" s="2" t="inlineStr">
+        <is>
+          <t>heatmap toggle -&gt; on</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -3644,8 +4176,16 @@
         </is>
       </c>
       <c r="H76" s="3" t="inlineStr"/>
-      <c r="I76" s="2" t="inlineStr"/>
-      <c r="J76" s="2" t="inlineStr"/>
+      <c r="I76" s="2" t="inlineStr">
+        <is>
+          <t>Needs Rig</t>
+        </is>
+      </c>
+      <c r="J76" s="2" t="inlineStr">
+        <is>
+          <t>move = เคลื่อนหุ่น</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -3686,7 +4226,11 @@
         </is>
       </c>
       <c r="H77" s="3" t="inlineStr"/>
-      <c r="I77" s="2" t="inlineStr"/>
+      <c r="I77" s="2" t="inlineStr">
+        <is>
+          <t>Needs Rig</t>
+        </is>
+      </c>
       <c r="J77" s="2" t="inlineStr"/>
     </row>
     <row r="78">
@@ -3727,7 +4271,11 @@
         </is>
       </c>
       <c r="H78" s="3" t="inlineStr"/>
-      <c r="I78" s="2" t="inlineStr"/>
+      <c r="I78" s="2" t="inlineStr">
+        <is>
+          <t>Needs Rig</t>
+        </is>
+      </c>
       <c r="J78" s="2" t="inlineStr"/>
     </row>
     <row r="79">
@@ -3769,7 +4317,11 @@
         </is>
       </c>
       <c r="H79" s="3" t="inlineStr"/>
-      <c r="I79" s="2" t="inlineStr"/>
+      <c r="I79" s="2" t="inlineStr">
+        <is>
+          <t>Needs Rig</t>
+        </is>
+      </c>
       <c r="J79" s="2" t="inlineStr"/>
     </row>
     <row r="80">
@@ -3810,8 +4362,16 @@
         </is>
       </c>
       <c r="H80" s="3" t="inlineStr"/>
-      <c r="I80" s="2" t="inlineStr"/>
-      <c r="J80" s="2" t="inlineStr"/>
+      <c r="I80" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J80" s="2" t="inlineStr">
+        <is>
+          <t>emergency-stop -&gt; triggered</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -3852,8 +4412,16 @@
         </is>
       </c>
       <c r="H81" s="3" t="inlineStr"/>
-      <c r="I81" s="2" t="inlineStr"/>
-      <c r="J81" s="2" t="inlineStr"/>
+      <c r="I81" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J81" s="2" t="inlineStr">
+        <is>
+          <t>GET settings 200</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -3894,8 +4462,16 @@
         </is>
       </c>
       <c r="H82" s="3" t="inlineStr"/>
-      <c r="I82" s="2" t="inlineStr"/>
-      <c r="J82" s="2" t="inlineStr"/>
+      <c r="I82" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J82" s="2" t="inlineStr">
+        <is>
+          <t>PUT + persist (key กลับมา)</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -3936,8 +4512,16 @@
         </is>
       </c>
       <c r="H83" s="3" t="inlineStr"/>
-      <c r="I83" s="2" t="inlineStr"/>
-      <c r="J83" s="2" t="inlineStr"/>
+      <c r="I83" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J83" s="2" t="inlineStr">
+        <is>
+          <t>key อื่นไม่โดนแก้</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -3977,8 +4561,16 @@
         </is>
       </c>
       <c r="H84" s="3" t="inlineStr"/>
-      <c r="I84" s="2" t="inlineStr"/>
-      <c r="J84" s="2" t="inlineStr"/>
+      <c r="I84" s="2" t="inlineStr">
+        <is>
+          <t>Needs Config</t>
+        </is>
+      </c>
+      <c r="J84" s="2" t="inlineStr">
+        <is>
+          <t>ต้องมี Blynk token</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -4018,7 +4610,11 @@
         </is>
       </c>
       <c r="H85" s="3" t="inlineStr"/>
-      <c r="I85" s="2" t="inlineStr"/>
+      <c r="I85" s="2" t="inlineStr">
+        <is>
+          <t>Needs Config</t>
+        </is>
+      </c>
       <c r="J85" s="2" t="inlineStr"/>
     </row>
     <row r="86">
@@ -4059,7 +4655,11 @@
         </is>
       </c>
       <c r="H86" s="3" t="inlineStr"/>
-      <c r="I86" s="2" t="inlineStr"/>
+      <c r="I86" s="2" t="inlineStr">
+        <is>
+          <t>Needs Config</t>
+        </is>
+      </c>
       <c r="J86" s="2" t="inlineStr"/>
     </row>
     <row r="87">
@@ -4101,8 +4701,16 @@
         </is>
       </c>
       <c r="H87" s="3" t="inlineStr"/>
-      <c r="I87" s="2" t="inlineStr"/>
-      <c r="J87" s="2" t="inlineStr"/>
+      <c r="I87" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J87" s="2" t="inlineStr">
+        <is>
+          <t>ping 200 (device unreachable=false result)</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -4143,8 +4751,16 @@
         </is>
       </c>
       <c r="H88" s="3" t="inlineStr"/>
-      <c r="I88" s="2" t="inlineStr"/>
-      <c r="J88" s="2" t="inlineStr"/>
+      <c r="I88" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J88" s="2" t="inlineStr">
+        <is>
+          <t>no token -&gt; 401</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -4185,8 +4801,16 @@
         </is>
       </c>
       <c r="H89" s="3" t="inlineStr"/>
-      <c r="I89" s="2" t="inlineStr"/>
-      <c r="J89" s="2" t="inlineStr"/>
+      <c r="I89" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J89" s="2" t="inlineStr">
+        <is>
+          <t>evil origin -&gt; ACAO none</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -4226,8 +4850,16 @@
         </is>
       </c>
       <c r="H90" s="3" t="inlineStr"/>
-      <c r="I90" s="2" t="inlineStr"/>
-      <c r="J90" s="2" t="inlineStr"/>
+      <c r="I90" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J90" s="2" t="inlineStr">
+        <is>
+          <t>OPTIONS -&gt; 405 (ไม่โดน 401)</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -4267,8 +4899,16 @@
         </is>
       </c>
       <c r="H91" s="3" t="inlineStr"/>
-      <c r="I91" s="2" t="inlineStr"/>
-      <c r="J91" s="2" t="inlineStr"/>
+      <c r="I91" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J91" s="2" t="inlineStr">
+        <is>
+          <t>backend root 200 message; หลัง nginx / = SPA (ปกติ)</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -4784,7 +5424,15 @@
       <c r="D2" t="n">
         <v>0</v>
       </c>
-      <c r="H2" t="inlineStr"/>
+      <c r="E2" t="n">
+        <v>12</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -4801,7 +5449,15 @@
       <c r="D3" t="n">
         <v>0</v>
       </c>
-      <c r="H3" t="inlineStr"/>
+      <c r="E3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -4818,7 +5474,15 @@
       <c r="D4" t="n">
         <v>0</v>
       </c>
-      <c r="H4" t="inlineStr"/>
+      <c r="E4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -4835,7 +5499,15 @@
       <c r="D5" t="n">
         <v>0</v>
       </c>
-      <c r="H5" t="inlineStr"/>
+      <c r="E5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4852,7 +5524,15 @@
       <c r="D6" t="n">
         <v>0</v>
       </c>
-      <c r="H6" t="inlineStr"/>
+      <c r="E6" t="n">
+        <v>7</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4869,7 +5549,15 @@
       <c r="D7" t="n">
         <v>0</v>
       </c>
-      <c r="H7" t="inlineStr"/>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4886,7 +5574,15 @@
       <c r="D8" t="n">
         <v>0</v>
       </c>
-      <c r="H8" t="inlineStr"/>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4903,7 +5599,15 @@
       <c r="D9" t="n">
         <v>0</v>
       </c>
-      <c r="H9" t="inlineStr"/>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4920,7 +5624,15 @@
       <c r="D10" t="n">
         <v>0</v>
       </c>
-      <c r="H10" t="inlineStr"/>
+      <c r="E10" t="n">
+        <v>3</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4937,7 +5649,15 @@
       <c r="D11" t="n">
         <v>0</v>
       </c>
-      <c r="H11" t="inlineStr"/>
+      <c r="E11" t="n">
+        <v>4</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4957,7 +5677,6 @@
       <c r="E12" t="n">
         <v>12</v>
       </c>
-      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -4975,15 +5694,14 @@
         <v>12</v>
       </c>
       <c r="E13" t="n">
-        <v>12</v>
+        <v>54</v>
       </c>
       <c r="F13" t="n">
         <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" t="inlineStr"/>
+        <v>48</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -5006,10 +5724,6 @@
           <t>Fail</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -5026,10 +5740,6 @@
       <c r="D16" t="n">
         <v>0</v>
       </c>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -5046,10 +5756,6 @@
       <c r="D17" t="n">
         <v>0</v>
       </c>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -5066,10 +5772,6 @@
       <c r="D18" t="n">
         <v>0</v>
       </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>